<commit_message>
feat: tambah kamus wording dan pilihan bahasa
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1775,15 +1775,19 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Waktu ditampilkan dalam WIB.</t>
+          <t>Waktu ditampilkan dalam {zona} ({namaZona}).</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Times are shown in WIB (UTC+7).</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr"/>
+          <t>Times are shown in {zone} (UTC{offset}).</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>{zona}/{zone} diisi WIB, WITA, atau WIT sesuai acara.</t>
+        </is>
+      </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
           <t>Draf</t>
@@ -2289,15 +2293,19 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Batas konfirmasi: {tanggal}, {jam} WIB.</t>
+          <t>Batas konfirmasi: {waktu}.</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>Please reply by {date}, {time} WIB.</t>
-        </is>
-      </c>
-      <c r="F47" s="8" t="inlineStr"/>
+          <t>Please reply by {when}.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>{waktu} berisi tanggal, jam, dan zona acara.</t>
+        </is>
+      </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
           <t>Draf</t>
@@ -5610,11 +5618,1337 @@
         </is>
       </c>
       <c r="H142" s="10" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="inlineStr">
+        <is>
+          <t>hero.facts</t>
+        </is>
+      </c>
+      <c r="B143" s="8" t="inlineStr">
+        <is>
+          <t>Pembuka</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>Label kartu waktu dan tempat</t>
+        </is>
+      </c>
+      <c r="D143" s="10" t="inlineStr">
+        <is>
+          <t>Catat pertemuannya</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="inlineStr">
+        <is>
+          <t>Save the date</t>
+        </is>
+      </c>
+      <c r="F143" s="8" t="n"/>
+      <c r="G143" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H143" s="10" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="inlineStr">
+        <is>
+          <t>hero.facts.aria</t>
+        </is>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>Pembuka</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D144" s="10" t="inlineStr">
+        <is>
+          <t>Waktu dan tempat acara</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="inlineStr">
+        <is>
+          <t>Date and venue</t>
+        </is>
+      </c>
+      <c r="F144" s="8" t="n"/>
+      <c r="G144" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H144" s="10" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="inlineStr">
+        <is>
+          <t>hero.date.empty</t>
+        </is>
+      </c>
+      <c r="B145" s="8" t="inlineStr">
+        <is>
+          <t>Pembuka</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>Bila tanggal kosong</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr">
+        <is>
+          <t>Tanggal belum diisi</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>Date to be confirmed</t>
+        </is>
+      </c>
+      <c r="F145" s="8" t="n"/>
+      <c r="G145" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H145" s="10" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="inlineStr">
+        <is>
+          <t>hero.place.empty</t>
+        </is>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>Pembuka</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>Bila tempat kosong</t>
+        </is>
+      </c>
+      <c r="D146" s="10" t="inlineStr">
+        <is>
+          <t>Lokasi belum ditentukan</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
+        <is>
+          <t>Venue to be confirmed</t>
+        </is>
+      </c>
+      <c r="F146" s="8" t="n"/>
+      <c r="G146" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H146" s="10" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="inlineStr">
+        <is>
+          <t>nav.prepare</t>
+        </is>
+      </c>
+      <c r="B147" s="8" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>Menu atas</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>Persiapan</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>Before you come</t>
+        </is>
+      </c>
+      <c r="F147" s="8" t="n"/>
+      <c r="G147" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H147" s="10" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="8" t="inlineStr">
+        <is>
+          <t>nav.label</t>
+        </is>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D148" s="10" t="inlineStr">
+        <is>
+          <t>Bagian undangan</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="inlineStr">
+        <is>
+          <t>Invitation sections</t>
+        </is>
+      </c>
+      <c r="F148" s="8" t="n"/>
+      <c r="G148" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H148" s="10" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="8" t="inlineStr">
+        <is>
+          <t>nav.top.aria</t>
+        </is>
+      </c>
+      <c r="B149" s="8" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Tombol bulat kembali ke atas</t>
+        </is>
+      </c>
+      <c r="D149" s="10" t="inlineStr">
+        <is>
+          <t>Kembali ke atas undangan</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="inlineStr">
+        <is>
+          <t>Back to the top of the invitation</t>
+        </is>
+      </c>
+      <c r="F149" s="8" t="n"/>
+      <c r="G149" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H149" s="10" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="8" t="inlineStr">
+        <is>
+          <t>shortcut.label</t>
+        </is>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>Pembuka</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D150" s="10" t="inlineStr">
+        <is>
+          <t>Pintasan undangan</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="inlineStr">
+        <is>
+          <t>Invitation shortcuts</t>
+        </is>
+      </c>
+      <c r="F150" s="8" t="n"/>
+      <c r="G150" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H150" s="10" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="8" t="inlineStr">
+        <is>
+          <t>section.about.title</t>
+        </is>
+      </c>
+      <c r="B151" s="8" t="inlineStr">
+        <is>
+          <t>Tentang acara</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>Judul bagian Tentang</t>
+        </is>
+      </c>
+      <c r="D151" s="10" t="inlineStr">
+        <is>
+          <t>Bertemu, berdiskusi, menyusun langkah bersama.</t>
+        </is>
+      </c>
+      <c r="E151" s="10" t="inlineStr">
+        <is>
+          <t>Meet, talk, and plan the next steps together.</t>
+        </is>
+      </c>
+      <c r="F151" s="8" t="n"/>
+      <c r="G151" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H151" s="10" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="8" t="inlineStr">
+        <is>
+          <t>section.about.topics</t>
+        </is>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>Tentang acara</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>Judul daftar topik</t>
+        </is>
+      </c>
+      <c r="D152" s="10" t="inlineStr">
+        <is>
+          <t>Pokok pembahasan</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="F152" s="8" t="n"/>
+      <c r="G152" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H152" s="10" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="8" t="inlineStr">
+        <is>
+          <t>section.prepare.title</t>
+        </is>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>Persiapan tamu</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>Judul bila kosong</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr">
+        <is>
+          <t>Yang perlu Anda ketahui sebelum datang.</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="inlineStr">
+        <is>
+          <t>Good to know before you come.</t>
+        </is>
+      </c>
+      <c r="F153" s="8" t="n"/>
+      <c r="G153" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H153" s="10" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="8" t="inlineStr">
+        <is>
+          <t>preview.notice</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>Pratinjau</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>Hanya di pratinjau admin</t>
+        </is>
+      </c>
+      <c r="D154" s="10" t="inlineStr">
+        <is>
+          <t>Pratinjau admin — undangan ini belum tentu dipublikasikan. Pengiriman RSVP dan survei dinonaktifkan.</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>Admin preview — this invitation may not be published yet. RSVP and survey sending are turned off.</t>
+        </is>
+      </c>
+      <c r="F154" s="8" t="n"/>
+      <c r="G154" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H154" s="10" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="8" t="inlineStr">
+        <is>
+          <t>common.newTab</t>
+        </is>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>Umum</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar, setelah tautan</t>
+        </is>
+      </c>
+      <c r="D155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (tab baru)</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (opens in a new tab)</t>
+        </is>
+      </c>
+      <c r="F155" s="8" t="n"/>
+      <c r="G155" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H155" s="10" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t>location.copyFailed</t>
+        </is>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>Bila salin gagal</t>
+        </is>
+      </c>
+      <c r="D156" s="10" t="inlineStr">
+        <is>
+          <t>Alamat belum dapat disalin. Pilih dan salin teks alamat di atas.</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="inlineStr">
+        <is>
+          <t>The address couldn't be copied. Please select and copy it above.</t>
+        </is>
+      </c>
+      <c r="F156" s="8" t="n"/>
+      <c r="G156" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H156" s="10" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="inlineStr">
+        <is>
+          <t>location.mapFailed</t>
+        </is>
+      </c>
+      <c r="B157" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>Bila peta gagal dimuat</t>
+        </is>
+      </c>
+      <c r="D157" s="10" t="inlineStr">
+        <is>
+          <t>Peta tidak dapat ditampilkan.</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="inlineStr">
+        <is>
+          <t>The map couldn't be shown.</t>
+        </is>
+      </c>
+      <c r="F157" s="8" t="n"/>
+      <c r="G157" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H157" s="10" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t>location.openMaps</t>
+        </is>
+      </c>
+      <c r="B158" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t>Tautan cadangan</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>Buka petunjuk lokasi di Google Maps</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
+        <is>
+          <t>Open directions in Google Maps</t>
+        </is>
+      </c>
+      <c r="F158" s="8" t="n"/>
+      <c r="G158" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H158" s="10" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="8" t="inlineStr">
+        <is>
+          <t>location.mapTitle</t>
+        </is>
+      </c>
+      <c r="B159" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>Judul peta untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D159" s="10" t="inlineStr">
+        <is>
+          <t>Peta lokasi {tempat}</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="inlineStr">
+        <is>
+          <t>Map of {place}</t>
+        </is>
+      </c>
+      <c r="F159" s="8" t="n"/>
+      <c r="G159" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H159" s="10" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t>location.photos</t>
+        </is>
+      </c>
+      <c r="B160" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t>Judul foto lokasi</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr">
+        <is>
+          <t>Foto lokasi {tempat}</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
+        <is>
+          <t>Photos of {place}</t>
+        </is>
+      </c>
+      <c r="F160" s="8" t="n"/>
+      <c r="G160" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H160" s="10" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="inlineStr">
+        <is>
+          <t>location.place.fallback</t>
+        </is>
+      </c>
+      <c r="B161" s="8" t="inlineStr">
+        <is>
+          <t>Lokasi</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t>Pengganti nama tempat yang kosong</t>
+        </is>
+      </c>
+      <c r="D161" s="10" t="inlineStr">
+        <is>
+          <t>acara</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t>the venue</t>
+        </is>
+      </c>
+      <c r="F161" s="8" t="n"/>
+      <c r="G161" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H161" s="10" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.locked</t>
+        </is>
+      </c>
+      <c r="B162" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>Tautan personal, RSVP terkunci</t>
+        </is>
+      </c>
+      <c r="D162" s="10" t="inlineStr">
+        <is>
+          <t>RSVP tersimpan: {jawaban}. Konfirmasi tidak dapat diubah saat ini.</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="inlineStr">
+        <is>
+          <t>Your reply: {answer}. It can't be changed at the moment.</t>
+        </is>
+      </c>
+      <c r="F162" s="8" t="n"/>
+      <c r="G162" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H162" s="10" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.answer.yes</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Isi {jawaban}</t>
+        </is>
+      </c>
+      <c r="D163" s="10" t="inlineStr">
+        <is>
+          <t>Hadir</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr">
+        <is>
+          <t>Attending</t>
+        </is>
+      </c>
+      <c r="F163" s="8" t="n"/>
+      <c r="G163" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H163" s="10" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.answer.no</t>
+        </is>
+      </c>
+      <c r="B164" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="inlineStr">
+        <is>
+          <t>Isi {jawaban}</t>
+        </is>
+      </c>
+      <c r="D164" s="10" t="inlineStr">
+        <is>
+          <t>Tidak hadir</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>Not attending</t>
+        </is>
+      </c>
+      <c r="F164" s="8" t="n"/>
+      <c r="G164" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H164" s="10" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.notOpen</t>
+        </is>
+      </c>
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t>Bila RSVP belum dibuka</t>
+        </is>
+      </c>
+      <c r="D165" s="10" t="inlineStr">
+        <is>
+          <t>Konfirmasi kehadiran belum dibuka oleh panitia.</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="inlineStr">
+        <is>
+          <t>RSVP hasn't opened yet.</t>
+        </is>
+      </c>
+      <c r="F165" s="8" t="n"/>
+      <c r="G165" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H165" s="10" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.noscript</t>
+        </is>
+      </c>
+      <c r="B166" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C166" s="8" t="inlineStr">
+        <is>
+          <t>Tanpa JavaScript</t>
+        </is>
+      </c>
+      <c r="D166" s="10" t="inlineStr">
+        <is>
+          <t>Aktifkan JavaScript untuk mengirim konfirmasi kehadiran.</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>Please turn on JavaScript to send your reply.</t>
+        </is>
+      </c>
+      <c r="F166" s="8" t="n"/>
+      <c r="G166" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H166" s="10" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>feedback.opensAt</t>
+        </is>
+      </c>
+      <c r="B167" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>Sebelum survei dibuka</t>
+        </is>
+      </c>
+      <c r="D167" s="10" t="inlineStr">
+        <is>
+          <t>Survei dibuka pada {waktu}.</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="inlineStr">
+        <is>
+          <t>The survey opens on {when}.</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="n"/>
+      <c r="G167" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H167" s="10" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
+          <t>feedback.noscript</t>
+        </is>
+      </c>
+      <c r="B168" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>Tanpa JavaScript</t>
+        </is>
+      </c>
+      <c r="D168" s="10" t="inlineStr">
+        <is>
+          <t>Aktifkan JavaScript untuk mengirim masukan.</t>
+        </is>
+      </c>
+      <c r="E168" s="10" t="inlineStr">
+        <is>
+          <t>Please turn on JavaScript to send feedback.</t>
+        </is>
+      </c>
+      <c r="F168" s="8" t="n"/>
+      <c r="G168" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H168" s="10" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="8" t="inlineStr">
+        <is>
+          <t>contact.whatsapp.aria</t>
+        </is>
+      </c>
+      <c r="B169" s="8" t="inlineStr">
+        <is>
+          <t>Kontak</t>
+        </is>
+      </c>
+      <c r="C169" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D169" s="10" t="inlineStr">
+        <is>
+          <t>Hubungi {nama} via WhatsApp</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="inlineStr">
+        <is>
+          <t>Chat with {name} on WhatsApp</t>
+        </is>
+      </c>
+      <c r="F169" s="8" t="n"/>
+      <c r="G169" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H169" s="10" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t>contact.call.aria</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>Kontak</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>Telepon {nama}</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="inlineStr">
+        <is>
+          <t>Call {name}</t>
+        </is>
+      </c>
+      <c r="F170" s="8" t="n"/>
+      <c r="G170" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H170" s="10" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="8" t="inlineStr">
+        <is>
+          <t>today.place.fallback</t>
+        </is>
+      </c>
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>Hari H</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t>Bila tempat kosong</t>
+        </is>
+      </c>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>Lokasi acara</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr">
+        <is>
+          <t>Event venue</t>
+        </is>
+      </c>
+      <c r="F171" s="8" t="n"/>
+      <c r="G171" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H171" s="10" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t>gallery.label</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D172" s="10" t="inlineStr">
+        <is>
+          <t>Foto lokasi</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="inlineStr">
+        <is>
+          <t>Venue photos</t>
+        </is>
+      </c>
+      <c r="F172" s="8" t="n"/>
+      <c r="G172" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H172" s="10" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="8" t="inlineStr">
+        <is>
+          <t>gallery.prev</t>
+        </is>
+      </c>
+      <c r="B173" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>Tombol panah</t>
+        </is>
+      </c>
+      <c r="D173" s="10" t="inlineStr">
+        <is>
+          <t>Foto sebelumnya</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="inlineStr">
+        <is>
+          <t>Previous photo</t>
+        </is>
+      </c>
+      <c r="F173" s="8" t="n"/>
+      <c r="G173" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H173" s="10" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t>gallery.next</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t>Tombol panah</t>
+        </is>
+      </c>
+      <c r="D174" s="10" t="inlineStr">
+        <is>
+          <t>Foto berikutnya</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="inlineStr">
+        <is>
+          <t>Next photo</t>
+        </is>
+      </c>
+      <c r="F174" s="8" t="n"/>
+      <c r="G174" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H174" s="10" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="8" t="inlineStr">
+        <is>
+          <t>gallery.pick</t>
+        </is>
+      </c>
+      <c r="B175" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D175" s="10" t="inlineStr">
+        <is>
+          <t>Pilih foto</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="inlineStr">
+        <is>
+          <t>Choose a photo</t>
+        </is>
+      </c>
+      <c r="F175" s="8" t="n"/>
+      <c r="G175" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H175" s="10" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="8" t="inlineStr">
+        <is>
+          <t>gallery.photo</t>
+        </is>
+      </c>
+      <c r="B176" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C176" s="8" t="inlineStr">
+        <is>
+          <t>Titik foto</t>
+        </is>
+      </c>
+      <c r="D176" s="10" t="inlineStr">
+        <is>
+          <t>Foto {n}</t>
+        </is>
+      </c>
+      <c r="E176" s="10" t="inlineStr">
+        <is>
+          <t>Photo {n}</t>
+        </is>
+      </c>
+      <c r="F176" s="8" t="n"/>
+      <c r="G176" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H176" s="10" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="8" t="inlineStr">
+        <is>
+          <t>gallery.position</t>
+        </is>
+      </c>
+      <c r="B177" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D177" s="10" t="inlineStr">
+        <is>
+          <t>{n} dari {total}</t>
+        </is>
+      </c>
+      <c r="E177" s="10" t="inlineStr">
+        <is>
+          <t>{n} of {total}</t>
+        </is>
+      </c>
+      <c r="F177" s="8" t="n"/>
+      <c r="G177" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H177" s="10" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="8" t="inlineStr">
+        <is>
+          <t>gallery.pause</t>
+        </is>
+      </c>
+      <c r="B178" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C178" s="8" t="inlineStr">
+        <is>
+          <t>Tombol putar otomatis</t>
+        </is>
+      </c>
+      <c r="D178" s="10" t="inlineStr">
+        <is>
+          <t>Hentikan pergantian otomatis</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="inlineStr">
+        <is>
+          <t>Pause the slideshow</t>
+        </is>
+      </c>
+      <c r="F178" s="8" t="n"/>
+      <c r="G178" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H178" s="10" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="8" t="inlineStr">
+        <is>
+          <t>gallery.play</t>
+        </is>
+      </c>
+      <c r="B179" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C179" s="8" t="inlineStr">
+        <is>
+          <t>Tombol putar otomatis</t>
+        </is>
+      </c>
+      <c r="D179" s="10" t="inlineStr">
+        <is>
+          <t>Jalankan pergantian otomatis</t>
+        </is>
+      </c>
+      <c r="E179" s="10" t="inlineStr">
+        <is>
+          <t>Play the slideshow</t>
+        </is>
+      </c>
+      <c r="F179" s="8" t="n"/>
+      <c r="G179" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H179" s="10" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="8" t="inlineStr">
+        <is>
+          <t>lang.label</t>
+        </is>
+      </c>
+      <c r="B180" s="8" t="inlineStr">
+        <is>
+          <t>Bahasa</t>
+        </is>
+      </c>
+      <c r="C180" s="8" t="inlineStr">
+        <is>
+          <t>Tombol bahasa, pembaca layar</t>
+        </is>
+      </c>
+      <c r="D180" s="10" t="inlineStr">
+        <is>
+          <t>Bahasa</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="F180" s="8" t="n"/>
+      <c r="G180" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H180" s="10" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="8" t="inlineStr">
+        <is>
+          <t>lang.fallback</t>
+        </is>
+      </c>
+      <c r="B181" s="8" t="inlineStr">
+        <is>
+          <t>Bahasa</t>
+        </is>
+      </c>
+      <c r="C181" s="8" t="inlineStr">
+        <is>
+          <t>Bila sebagian isi belum diterjemahkan</t>
+        </is>
+      </c>
+      <c r="D181" s="10" t="inlineStr">
+        <is>
+          <t>Sebagian informasi hanya tersedia dalam Bahasa Indonesia.</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="inlineStr">
+        <is>
+          <t>Some details are only available in Indonesian.</t>
+        </is>
+      </c>
+      <c r="F181" s="8" t="n"/>
+      <c r="G181" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H181" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8272,7 +9606,7 @@
   </sheetData>
   <autoFilter ref="A1:H76"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: tambah impor tamu, kirim WhatsApp, dan status dibuka
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H181"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6945,10 +6945,124 @@
       </c>
       <c r="H181" s="10" t="n"/>
     </row>
+    <row r="182">
+      <c r="A182" s="8" t="inlineStr">
+        <is>
+          <t>wa.invite</t>
+        </is>
+      </c>
+      <c r="B182" s="8" t="inlineStr">
+        <is>
+          <t>Pesan WhatsApp</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="inlineStr">
+        <is>
+          <t>Undangan, dikirim panitia lewat tombol Kirim WA</t>
+        </is>
+      </c>
+      <c r="D182" s="10" t="inlineStr">
+        <is>
+          <t>Halo {nama}, dengan senang hati kami mengundang Anda ke {acara} pada {waktu}. Undangan dan konfirmasi kehadiran ada di tautan pribadi ini: {tautan}</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="inlineStr">
+        <is>
+          <t>Hello {name}, we are delighted to invite you to {event} on {when}. Your invitation and RSVP are at this personal link: {link}</t>
+        </is>
+      </c>
+      <c r="F182" s="8" t="inlineStr">
+        <is>
+          <t>{nama}, {acara}, {waktu}, {batas}, dan {tautan} diisi otomatis.</t>
+        </is>
+      </c>
+      <c r="G182" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H182" s="10" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="8" t="inlineStr">
+        <is>
+          <t>wa.reminder</t>
+        </is>
+      </c>
+      <c r="B183" s="8" t="inlineStr">
+        <is>
+          <t>Pesan WhatsApp</t>
+        </is>
+      </c>
+      <c r="C183" s="8" t="inlineStr">
+        <is>
+          <t>Pengingat untuk tamu yang belum menjawab, bila ada batas RSVP</t>
+        </is>
+      </c>
+      <c r="D183" s="10" t="inlineStr">
+        <is>
+          <t>Halo {nama}, sekadar mengingatkan: mohon konfirmasi kehadiran Anda untuk {acara} sebelum {batas}. Tautan undangan Anda: {tautan}</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="inlineStr">
+        <is>
+          <t>Hello {name}, a gentle reminder to confirm your attendance for {event} by {deadline}. Your invitation link: {link}</t>
+        </is>
+      </c>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>{nama}, {acara}, {waktu}, {batas}, dan {tautan} diisi otomatis.</t>
+        </is>
+      </c>
+      <c r="G183" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H183" s="10" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="8" t="inlineStr">
+        <is>
+          <t>wa.reminder.open</t>
+        </is>
+      </c>
+      <c r="B184" s="8" t="inlineStr">
+        <is>
+          <t>Pesan WhatsApp</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t>Pengingat bila tidak ada batas RSVP</t>
+        </is>
+      </c>
+      <c r="D184" s="10" t="inlineStr">
+        <is>
+          <t>Halo {nama}, sekadar mengingatkan: mohon konfirmasi kehadiran Anda untuk {acara} pada {waktu}. Tautan undangan Anda: {tautan}</t>
+        </is>
+      </c>
+      <c r="E184" s="10" t="inlineStr">
+        <is>
+          <t>Hello {name}, a gentle reminder to confirm your attendance for {event} on {when}. Your invitation link: {link}</t>
+        </is>
+      </c>
+      <c r="F184" s="8" t="inlineStr">
+        <is>
+          <t>{nama}, {acara}, {waktu}, {batas}, dan {tautan} diisi otomatis.</t>
+        </is>
+      </c>
+      <c r="G184" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H184" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: ubah RSVP menjadi form bertahap dengan kebutuhan tamu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H184"/>
+  <dimension ref="A1:H212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2713,15 +2713,19 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Langkah {n} dari 4</t>
+          <t>Langkah {n} dari {total}</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>Step {n} of 4</t>
-        </is>
-      </c>
-      <c r="F59" s="8" t="inlineStr"/>
+          <t>Step {n} of {total}</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>Tamu yang tidak hadir melewati langkah kebutuhan, jadi jumlah langkahnya 3.</t>
+        </is>
+      </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
           <t>Draf</t>
@@ -7058,11 +7062,963 @@
         </is>
       </c>
       <c r="H184" s="10" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.s1.titleOpen</t>
+        </is>
+      </c>
+      <c r="B185" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C185" s="8" t="inlineStr">
+        <is>
+          <t>Langkah 1, tautan umum</t>
+        </is>
+      </c>
+      <c r="D185" s="10" t="inlineStr">
+        <is>
+          <t>Apakah Anda bisa hadir?</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="inlineStr">
+        <is>
+          <t>Will you be able to join us?</t>
+        </is>
+      </c>
+      <c r="F185" s="8" t="n"/>
+      <c r="G185" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H185" s="10" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.party.label</t>
+        </is>
+      </c>
+      <c r="B186" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="inlineStr">
+        <is>
+          <t>Langkah 1, bila boleh membawa pendamping</t>
+        </is>
+      </c>
+      <c r="D186" s="10" t="inlineStr">
+        <is>
+          <t>Berapa orang yang datang bersama Anda?</t>
+        </is>
+      </c>
+      <c r="E186" s="10" t="inlineStr">
+        <is>
+          <t>How many people are coming with you?</t>
+        </is>
+      </c>
+      <c r="F186" s="8" t="n"/>
+      <c r="G186" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H186" s="10" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.party.hint</t>
+        </is>
+      </c>
+      <c r="B187" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah pilihan pendamping</t>
+        </is>
+      </c>
+      <c r="D187" s="10" t="inlineStr">
+        <is>
+          <t>Undangan ini berlaku untuk Anda dan paling banyak {n} pendamping.</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="inlineStr">
+        <is>
+          <t>This invitation covers you and up to {n} companions.</t>
+        </is>
+      </c>
+      <c r="F187" s="8" t="n"/>
+      <c r="G187" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H187" s="10" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.party.none</t>
+        </is>
+      </c>
+      <c r="B188" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C188" s="8" t="inlineStr">
+        <is>
+          <t>Pilihan pendamping</t>
+        </is>
+      </c>
+      <c r="D188" s="10" t="inlineStr">
+        <is>
+          <t>Datang sendiri</t>
+        </is>
+      </c>
+      <c r="E188" s="10" t="inlineStr">
+        <is>
+          <t>Just me</t>
+        </is>
+      </c>
+      <c r="F188" s="8" t="n"/>
+      <c r="G188" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H188" s="10" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.party.count</t>
+        </is>
+      </c>
+      <c r="B189" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C189" s="8" t="inlineStr">
+        <is>
+          <t>Pilihan pendamping</t>
+        </is>
+      </c>
+      <c r="D189" s="10" t="inlineStr">
+        <is>
+          <t>+{n} pendamping</t>
+        </is>
+      </c>
+      <c r="E189" s="10" t="inlineStr">
+        <is>
+          <t>+{n} companion(s)</t>
+        </is>
+      </c>
+      <c r="F189" s="8" t="n"/>
+      <c r="G189" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H189" s="10" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.companion.name</t>
+        </is>
+      </c>
+      <c r="B190" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C190" s="8" t="inlineStr">
+        <is>
+          <t>Kolom nama pendamping</t>
+        </is>
+      </c>
+      <c r="D190" s="10" t="inlineStr">
+        <is>
+          <t>Nama pendamping {n} (opsional)</t>
+        </is>
+      </c>
+      <c r="E190" s="10" t="inlineStr">
+        <is>
+          <t>Companion {n} name (optional)</t>
+        </is>
+      </c>
+      <c r="F190" s="8" t="n"/>
+      <c r="G190" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H190" s="10" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="8" t="inlineStr">
+        <is>
+          <t>need.interpreter</t>
+        </is>
+      </c>
+      <c r="B191" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C191" s="8" t="inlineStr">
+        <is>
+          <t>Pilihan akses</t>
+        </is>
+      </c>
+      <c r="D191" s="10" t="inlineStr">
+        <is>
+          <t>Juru bahasa isyarat</t>
+        </is>
+      </c>
+      <c r="E191" s="10" t="inlineStr">
+        <is>
+          <t>Sign language interpreter</t>
+        </is>
+      </c>
+      <c r="F191" s="8" t="n"/>
+      <c r="G191" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H191" s="10" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="8" t="inlineStr">
+        <is>
+          <t>need.other.detail</t>
+        </is>
+      </c>
+      <c r="B192" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C192" s="8" t="inlineStr">
+        <is>
+          <t>Kolom bila memilih Lainnya</t>
+        </is>
+      </c>
+      <c r="D192" s="10" t="inlineStr">
+        <is>
+          <t>Jelaskan singkat</t>
+        </is>
+      </c>
+      <c r="E192" s="10" t="inlineStr">
+        <is>
+          <t>Please describe briefly</t>
+        </is>
+      </c>
+      <c r="F192" s="8" t="n"/>
+      <c r="G192" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H192" s="10" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="8" t="inlineStr">
+        <is>
+          <t>field.whatsappConsent</t>
+        </is>
+      </c>
+      <c r="B193" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C193" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah nomor WhatsApp</t>
+        </is>
+      </c>
+      <c r="D193" s="10" t="inlineStr">
+        <is>
+          <t>Boleh dihubungi lewat WhatsApp untuk informasi acara ini.</t>
+        </is>
+      </c>
+      <c r="E193" s="10" t="inlineStr">
+        <is>
+          <t>You may contact me on WhatsApp about this event.</t>
+        </is>
+      </c>
+      <c r="F193" s="8" t="n"/>
+      <c r="G193" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H193" s="10" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.attendance</t>
+        </is>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C194" s="8" t="inlineStr">
+        <is>
+          <t>Ringkasan langkah 4</t>
+        </is>
+      </c>
+      <c r="D194" s="10" t="inlineStr">
+        <is>
+          <t>Kehadiran</t>
+        </is>
+      </c>
+      <c r="E194" s="10" t="inlineStr">
+        <is>
+          <t>Attendance</t>
+        </is>
+      </c>
+      <c r="F194" s="8" t="n"/>
+      <c r="G194" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H194" s="10" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.party</t>
+        </is>
+      </c>
+      <c r="B195" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C195" s="8" t="inlineStr">
+        <is>
+          <t>Ringkasan langkah 4</t>
+        </is>
+      </c>
+      <c r="D195" s="10" t="inlineStr">
+        <is>
+          <t>Rombongan</t>
+        </is>
+      </c>
+      <c r="E195" s="10" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="F195" s="8" t="n"/>
+      <c r="G195" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H195" s="10" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.partySize</t>
+        </is>
+      </c>
+      <c r="B196" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C196" s="8" t="inlineStr">
+        <is>
+          <t>Isi ringkasan rombongan</t>
+        </is>
+      </c>
+      <c r="D196" s="10" t="inlineStr">
+        <is>
+          <t>{n} orang</t>
+        </is>
+      </c>
+      <c r="E196" s="10" t="inlineStr">
+        <is>
+          <t>{n} people</t>
+        </is>
+      </c>
+      <c r="F196" s="8" t="n"/>
+      <c r="G196" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H196" s="10" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.details</t>
+        </is>
+      </c>
+      <c r="B197" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C197" s="8" t="inlineStr">
+        <is>
+          <t>Ringkasan langkah 4</t>
+        </is>
+      </c>
+      <c r="D197" s="10" t="inlineStr">
+        <is>
+          <t>Data diri</t>
+        </is>
+      </c>
+      <c r="E197" s="10" t="inlineStr">
+        <is>
+          <t>Your details</t>
+        </is>
+      </c>
+      <c r="F197" s="8" t="n"/>
+      <c r="G197" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H197" s="10" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.needs</t>
+        </is>
+      </c>
+      <c r="B198" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C198" s="8" t="inlineStr">
+        <is>
+          <t>Ringkasan langkah 4</t>
+        </is>
+      </c>
+      <c r="D198" s="10" t="inlineStr">
+        <is>
+          <t>Kebutuhan</t>
+        </is>
+      </c>
+      <c r="E198" s="10" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="F198" s="8" t="n"/>
+      <c r="G198" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H198" s="10" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.review.none</t>
+        </is>
+      </c>
+      <c r="B199" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C199" s="8" t="inlineStr">
+        <is>
+          <t>Bila tidak ada kebutuhan</t>
+        </is>
+      </c>
+      <c r="D199" s="10" t="inlineStr">
+        <is>
+          <t>Tidak ada kebutuhan khusus</t>
+        </is>
+      </c>
+      <c r="E199" s="10" t="inlineStr">
+        <is>
+          <t>No special requirements</t>
+        </is>
+      </c>
+      <c r="F199" s="8" t="n"/>
+      <c r="G199" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H199" s="10" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.privacy</t>
+        </is>
+      </c>
+      <c r="B200" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C200" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah persetujuan</t>
+        </is>
+      </c>
+      <c r="D200" s="10" t="inlineStr">
+        <is>
+          <t>Jawaban dan kebutuhan Anda hanya dilihat panitia untuk menyiapkan acara.</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="inlineStr">
+        <is>
+          <t>Your answers are only seen by the organisers to prepare the event.</t>
+        </is>
+      </c>
+      <c r="F200" s="8" t="n"/>
+      <c r="G200" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H200" s="10" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.saved.personal</t>
+        </is>
+      </c>
+      <c r="B201" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C201" s="8" t="inlineStr">
+        <is>
+          <t>Setelah terkirim, tautan personal</t>
+        </is>
+      </c>
+      <c r="D201" s="10" t="inlineStr">
+        <is>
+          <t>Buka kembali tautan ini untuk mengubah jawaban sampai batas konfirmasi.</t>
+        </is>
+      </c>
+      <c r="E201" s="10" t="inlineStr">
+        <is>
+          <t>Open this link again to change your reply until the RSVP deadline.</t>
+        </is>
+      </c>
+      <c r="F201" s="8" t="n"/>
+      <c r="G201" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H201" s="10" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.saved.open</t>
+        </is>
+      </c>
+      <c r="B202" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C202" s="8" t="inlineStr">
+        <is>
+          <t>Setelah terkirim, tautan umum</t>
+        </is>
+      </c>
+      <c r="D202" s="10" t="inlineStr">
+        <is>
+          <t>Terima kasih. Jawaban tidak disimpan di browser ini.</t>
+        </is>
+      </c>
+      <c r="E202" s="10" t="inlineStr">
+        <is>
+          <t>Thank you. Your reply isn't stored in this browser.</t>
+        </is>
+      </c>
+      <c r="F202" s="8" t="n"/>
+      <c r="G202" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H202" s="10" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.personal.note</t>
+        </is>
+      </c>
+      <c r="B203" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C203" s="8" t="inlineStr">
+        <is>
+          <t>Di kartu, tautan personal</t>
+        </is>
+      </c>
+      <c r="D203" s="10" t="inlineStr">
+        <is>
+          <t>Tautan ini khusus untuk Anda. Siapa pun yang memegangnya dapat melihat dan mengubah jawaban, jadi jangan dibagikan.</t>
+        </is>
+      </c>
+      <c r="E203" s="10" t="inlineStr">
+        <is>
+          <t>This link is just for you. Anyone holding it can see and change your reply, so please don't share it.</t>
+        </is>
+      </c>
+      <c r="F203" s="8" t="n"/>
+      <c r="G203" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H203" s="10" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="8" t="inlineStr">
+        <is>
+          <t>rsvp.closedNow</t>
+        </is>
+      </c>
+      <c r="B204" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C204" s="8" t="inlineStr">
+        <is>
+          <t>Bila ditutup saat mengisi</t>
+        </is>
+      </c>
+      <c r="D204" s="10" t="inlineStr">
+        <is>
+          <t>Konfirmasi kehadiran sudah ditutup.</t>
+        </is>
+      </c>
+      <c r="E204" s="10" t="inlineStr">
+        <is>
+          <t>RSVP has closed.</t>
+        </is>
+      </c>
+      <c r="F204" s="8" t="n"/>
+      <c r="G204" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H204" s="10" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="8" t="inlineStr">
+        <is>
+          <t>form.error.other</t>
+        </is>
+      </c>
+      <c r="B205" s="8" t="inlineStr">
+        <is>
+          <t>Konfirmasi</t>
+        </is>
+      </c>
+      <c r="C205" s="8" t="inlineStr">
+        <is>
+          <t>Kolom Lainnya kosong</t>
+        </is>
+      </c>
+      <c r="D205" s="10" t="inlineStr">
+        <is>
+          <t>Jelaskan kebutuhan lainnya.</t>
+        </is>
+      </c>
+      <c r="E205" s="10" t="inlineStr">
+        <is>
+          <t>Please describe the other requirement.</t>
+        </is>
+      </c>
+      <c r="F205" s="8" t="n"/>
+      <c r="G205" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H205" s="10" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="8" t="inlineStr">
+        <is>
+          <t>feedback.card.meta</t>
+        </is>
+      </c>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C206" s="8" t="inlineStr">
+        <is>
+          <t>Kartu survei</t>
+        </is>
+      </c>
+      <c r="D206" s="10" t="inlineStr">
+        <is>
+          <t>Sekitar 2 menit · tanpa nama</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="inlineStr">
+        <is>
+          <t>About 2 minutes · anonymous</t>
+        </is>
+      </c>
+      <c r="F206" s="8" t="n"/>
+      <c r="G206" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H206" s="10" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="8" t="inlineStr">
+        <is>
+          <t>feedback.card.start</t>
+        </is>
+      </c>
+      <c r="B207" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C207" s="8" t="inlineStr">
+        <is>
+          <t>Tombol kartu survei</t>
+        </is>
+      </c>
+      <c r="D207" s="10" t="inlineStr">
+        <is>
+          <t>Mulai survei</t>
+        </is>
+      </c>
+      <c r="E207" s="10" t="inlineStr">
+        <is>
+          <t>Start the survey</t>
+        </is>
+      </c>
+      <c r="F207" s="8" t="n"/>
+      <c r="G207" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H207" s="10" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="8" t="inlineStr">
+        <is>
+          <t>feedback.send</t>
+        </is>
+      </c>
+      <c r="B208" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C208" s="8" t="inlineStr">
+        <is>
+          <t>Tombol kirim survei</t>
+        </is>
+      </c>
+      <c r="D208" s="10" t="inlineStr">
+        <is>
+          <t>Kirim masukan</t>
+        </is>
+      </c>
+      <c r="E208" s="10" t="inlineStr">
+        <is>
+          <t>Send feedback</t>
+        </is>
+      </c>
+      <c r="F208" s="8" t="n"/>
+      <c r="G208" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H208" s="10" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="8" t="inlineStr">
+        <is>
+          <t>feedback.required</t>
+        </is>
+      </c>
+      <c r="B209" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C209" s="8" t="inlineStr">
+        <is>
+          <t>Di label pertanyaan</t>
+        </is>
+      </c>
+      <c r="D209" s="10" t="inlineStr">
+        <is>
+          <t>(wajib)</t>
+        </is>
+      </c>
+      <c r="E209" s="10" t="inlineStr">
+        <is>
+          <t>(required)</t>
+        </is>
+      </c>
+      <c r="F209" s="8" t="n"/>
+      <c r="G209" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H209" s="10" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="8" t="inlineStr">
+        <is>
+          <t>feedback.optional</t>
+        </is>
+      </c>
+      <c r="B210" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C210" s="8" t="inlineStr">
+        <is>
+          <t>Di label pertanyaan</t>
+        </is>
+      </c>
+      <c r="D210" s="10" t="inlineStr">
+        <is>
+          <t>(opsional)</t>
+        </is>
+      </c>
+      <c r="E210" s="10" t="inlineStr">
+        <is>
+          <t>(optional)</t>
+        </is>
+      </c>
+      <c r="F210" s="8" t="n"/>
+      <c r="G210" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H210" s="10" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="8" t="inlineStr">
+        <is>
+          <t>feedback.choose</t>
+        </is>
+      </c>
+      <c r="B211" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C211" s="8" t="inlineStr">
+        <is>
+          <t>Pilihan kosong</t>
+        </is>
+      </c>
+      <c r="D211" s="10" t="inlineStr">
+        <is>
+          <t>Pilih jawaban</t>
+        </is>
+      </c>
+      <c r="E211" s="10" t="inlineStr">
+        <is>
+          <t>Choose an answer</t>
+        </is>
+      </c>
+      <c r="F211" s="8" t="n"/>
+      <c r="G211" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H211" s="10" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="8" t="inlineStr">
+        <is>
+          <t>feedback.closedNow</t>
+        </is>
+      </c>
+      <c r="B212" s="8" t="inlineStr">
+        <is>
+          <t>Survei</t>
+        </is>
+      </c>
+      <c r="C212" s="8" t="inlineStr">
+        <is>
+          <t>Bila survei ditutup saat mengisi</t>
+        </is>
+      </c>
+      <c r="D212" s="10" t="inlineStr">
+        <is>
+          <t>Survei belum menerima jawaban saat ini.</t>
+        </is>
+      </c>
+      <c r="E212" s="10" t="inlineStr">
+        <is>
+          <t>The survey isn't accepting answers right now.</t>
+        </is>
+      </c>
+      <c r="F212" s="8" t="n"/>
+      <c r="G212" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H212" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: tambah jadwal per hari, detail kegiatan, dan kontak darurat
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H212"/>
+  <dimension ref="A1:H223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8015,10 +8015,384 @@
       </c>
       <c r="H212" s="10" t="n"/>
     </row>
+    <row r="213">
+      <c r="A213" s="8" t="inlineStr">
+        <is>
+          <t>program.tab</t>
+        </is>
+      </c>
+      <c r="B213" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C213" s="8" t="inlineStr">
+        <is>
+          <t>Tab hari di jadwal</t>
+        </is>
+      </c>
+      <c r="D213" s="10" t="inlineStr">
+        <is>
+          <t>Hari {n}</t>
+        </is>
+      </c>
+      <c r="E213" s="10" t="inlineStr">
+        <is>
+          <t>Day {n}</t>
+        </is>
+      </c>
+      <c r="F213" s="8" t="n"/>
+      <c r="G213" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H213" s="10" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="8" t="inlineStr">
+        <is>
+          <t>program.tabs.label</t>
+        </is>
+      </c>
+      <c r="B214" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C214" s="8" t="inlineStr">
+        <is>
+          <t>Untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D214" s="10" t="inlineStr">
+        <is>
+          <t>Pilih hari</t>
+        </is>
+      </c>
+      <c r="E214" s="10" t="inlineStr">
+        <is>
+          <t>Choose a day</t>
+        </is>
+      </c>
+      <c r="F214" s="8" t="n"/>
+      <c r="G214" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H214" s="10" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="8" t="inlineStr">
+        <is>
+          <t>detail.less</t>
+        </is>
+      </c>
+      <c r="B215" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C215" s="8" t="inlineStr">
+        <is>
+          <t>Tutup detail kegiatan</t>
+        </is>
+      </c>
+      <c r="D215" s="10" t="inlineStr">
+        <is>
+          <t>Tutup</t>
+        </is>
+      </c>
+      <c r="E215" s="10" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="F215" s="8" t="n"/>
+      <c r="G215" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H215" s="10" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="8" t="inlineStr">
+        <is>
+          <t>detail.moreLess</t>
+        </is>
+      </c>
+      <c r="B216" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C216" s="8" t="inlineStr">
+        <is>
+          <t>Sembunyikan cerita lengkap</t>
+        </is>
+      </c>
+      <c r="D216" s="10" t="inlineStr">
+        <is>
+          <t>Ringkas</t>
+        </is>
+      </c>
+      <c r="E216" s="10" t="inlineStr">
+        <is>
+          <t>Show less</t>
+        </is>
+      </c>
+      <c r="F216" s="8" t="n"/>
+      <c r="G216" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H216" s="10" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="8" t="inlineStr">
+        <is>
+          <t>duration.hours</t>
+        </is>
+      </c>
+      <c r="B217" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C217" s="8" t="inlineStr">
+        <is>
+          <t>Lama kegiatan</t>
+        </is>
+      </c>
+      <c r="D217" s="10" t="inlineStr">
+        <is>
+          <t>{n} jam</t>
+        </is>
+      </c>
+      <c r="E217" s="10" t="inlineStr">
+        <is>
+          <t>{n} h</t>
+        </is>
+      </c>
+      <c r="F217" s="8" t="n"/>
+      <c r="G217" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H217" s="10" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="8" t="inlineStr">
+        <is>
+          <t>duration.minutes</t>
+        </is>
+      </c>
+      <c r="B218" s="8" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C218" s="8" t="inlineStr">
+        <is>
+          <t>Lama kegiatan</t>
+        </is>
+      </c>
+      <c r="D218" s="10" t="inlineStr">
+        <is>
+          <t>{n} menit</t>
+        </is>
+      </c>
+      <c r="E218" s="10" t="inlineStr">
+        <is>
+          <t>{n} min</t>
+        </is>
+      </c>
+      <c r="F218" s="8" t="n"/>
+      <c r="G218" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H218" s="10" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="8" t="inlineStr">
+        <is>
+          <t>emergency.title</t>
+        </is>
+      </c>
+      <c r="B219" s="8" t="inlineStr">
+        <is>
+          <t>Kontak darurat</t>
+        </is>
+      </c>
+      <c r="C219" s="8" t="inlineStr">
+        <is>
+          <t>Judul kartu</t>
+        </is>
+      </c>
+      <c r="D219" s="10" t="inlineStr">
+        <is>
+          <t>Kontak darurat</t>
+        </is>
+      </c>
+      <c r="E219" s="10" t="inlineStr">
+        <is>
+          <t>Emergency contact</t>
+        </is>
+      </c>
+      <c r="F219" s="8" t="n"/>
+      <c r="G219" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H219" s="10" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="8" t="inlineStr">
+        <is>
+          <t>emergency.call</t>
+        </is>
+      </c>
+      <c r="B220" s="8" t="inlineStr">
+        <is>
+          <t>Kontak darurat</t>
+        </is>
+      </c>
+      <c r="C220" s="8" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D220" s="10" t="inlineStr">
+        <is>
+          <t>Telepon {name}</t>
+        </is>
+      </c>
+      <c r="E220" s="10" t="inlineStr">
+        <is>
+          <t>Call {name}</t>
+        </is>
+      </c>
+      <c r="F220" s="8" t="n"/>
+      <c r="G220" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H220" s="10" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="8" t="inlineStr">
+        <is>
+          <t>emergency.hospital</t>
+        </is>
+      </c>
+      <c r="B221" s="8" t="inlineStr">
+        <is>
+          <t>Kontak darurat</t>
+        </is>
+      </c>
+      <c r="C221" s="8" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D221" s="10" t="inlineStr">
+        <is>
+          <t>Rumah sakit terdekat</t>
+        </is>
+      </c>
+      <c r="E221" s="10" t="inlineStr">
+        <is>
+          <t>Nearest hospital</t>
+        </is>
+      </c>
+      <c r="F221" s="8" t="n"/>
+      <c r="G221" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H221" s="10" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="8" t="inlineStr">
+        <is>
+          <t>emergency.directions</t>
+        </is>
+      </c>
+      <c r="B222" s="8" t="inlineStr">
+        <is>
+          <t>Kontak darurat</t>
+        </is>
+      </c>
+      <c r="C222" s="8" t="inlineStr">
+        <is>
+          <t>Tautan</t>
+        </is>
+      </c>
+      <c r="D222" s="10" t="inlineStr">
+        <is>
+          <t>Petunjuk arah</t>
+        </is>
+      </c>
+      <c r="E222" s="10" t="inlineStr">
+        <is>
+          <t>Directions</t>
+        </is>
+      </c>
+      <c r="F222" s="8" t="n"/>
+      <c r="G222" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H222" s="10" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="8" t="inlineStr">
+        <is>
+          <t>offline.ready</t>
+        </is>
+      </c>
+      <c r="B223" s="8" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C223" s="8" t="inlineStr">
+        <is>
+          <t>Setelah halaman tersimpan</t>
+        </is>
+      </c>
+      <c r="D223" s="10" t="inlineStr">
+        <is>
+          <t>Halaman ini tersimpan di perangkat dan tetap bisa dibuka tanpa sinyal.</t>
+        </is>
+      </c>
+      <c r="E223" s="10" t="inlineStr">
+        <is>
+          <t>This page is saved on your device and opens without a signal.</t>
+        </is>
+      </c>
+      <c r="F223" s="8" t="n"/>
+      <c r="G223" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H223" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: tambah kalender, pratinjau tautan, QR undangan, dan sambutan beranda
- Berkas kalender .ics per sesi dengan pengingat 15/30/60 menit dan pilihan hari ini saja
- Kartu "Berikutnya · N menit lagi" di halaman Hari H
- Gambar pratinjau WhatsApp per acara tanpa nama tamu, serta metadataBase
- Kartu tautan umum dan unduhan QR PNG/SVG di halaman Undangan tamu
- Halaman depan berisi sambutan umum saat tidak ada acara tayang

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H223"/>
+  <dimension ref="A1:H225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8389,10 +8389,78 @@
       </c>
       <c r="H223" s="10" t="n"/>
     </row>
+    <row r="224">
+      <c r="A224" s="8" t="inlineStr">
+        <is>
+          <t>calendar.scope</t>
+        </is>
+      </c>
+      <c r="B224" s="8" t="inlineStr">
+        <is>
+          <t>Kalender</t>
+        </is>
+      </c>
+      <c r="C224" s="8" t="inlineStr">
+        <is>
+          <t>Judul pilihan</t>
+        </is>
+      </c>
+      <c r="D224" s="10" t="inlineStr">
+        <is>
+          <t>Yang disimpan</t>
+        </is>
+      </c>
+      <c r="E224" s="10" t="inlineStr">
+        <is>
+          <t>What to save</t>
+        </is>
+      </c>
+      <c r="F224" s="8" t="n"/>
+      <c r="G224" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H224" s="10" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="8" t="inlineStr">
+        <is>
+          <t>calendar.reminder</t>
+        </is>
+      </c>
+      <c r="B225" s="8" t="inlineStr">
+        <is>
+          <t>Kalender</t>
+        </is>
+      </c>
+      <c r="C225" s="8" t="inlineStr">
+        <is>
+          <t>Judul pilihan</t>
+        </is>
+      </c>
+      <c r="D225" s="10" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="E225" s="10" t="inlineStr">
+        <is>
+          <t>Reminder</t>
+        </is>
+      </c>
+      <c r="F225" s="8" t="n"/>
+      <c r="G225" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H225" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G223" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: tambah galeri foto acara di R2 dengan tinjauan sebelum tayang
- Unggah banyak foto: versi tampilan dan thumbnail WebP dibuat di browser, lalu langsung ke R2
- Alamat unggah bertanda tangan dengan tipe dan ukuran terkunci, serta pemeriksaan isi berkas
- Tinjau foto (menunggu, tayang, disembunyikan), keterangan, dan hapus
- Halaman galeri tamu dengan unduh asli dan minta hapus lewat WhatsApp PIC; tutup enam bulan setelah acara
- Mode "penyimpanan belum disiapkan" selama variabel R2 belum diisi
- Migrasi 202610210002_gallery_photos.sql beserta uji SQL lokal dan panduan bucket

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H225"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8457,10 +8457,282 @@
       </c>
       <c r="H225" s="10" t="n"/>
     </row>
+    <row r="226">
+      <c r="A226" s="8" t="inlineStr">
+        <is>
+          <t>photos.title</t>
+        </is>
+      </c>
+      <c r="B226" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C226" s="8" t="inlineStr">
+        <is>
+          <t>Judul halaman</t>
+        </is>
+      </c>
+      <c r="D226" s="10" t="inlineStr">
+        <is>
+          <t>Galeri foto acara</t>
+        </is>
+      </c>
+      <c r="E226" s="10" t="inlineStr">
+        <is>
+          <t>Event photos</t>
+        </is>
+      </c>
+      <c r="F226" s="8" t="n"/>
+      <c r="G226" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H226" s="10" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="8" t="inlineStr">
+        <is>
+          <t>photos.intro</t>
+        </is>
+      </c>
+      <c r="B227" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C227" s="8" t="inlineStr">
+        <is>
+          <t>Pengantar</t>
+        </is>
+      </c>
+      <c r="D227" s="10" t="inlineStr">
+        <is>
+          <t>Terima kasih sudah hadir. Simpan foto favorit Anda; ketuk foto untuk melihat lebih besar dan mengunduh versi aslinya.</t>
+        </is>
+      </c>
+      <c r="E227" s="10" t="inlineStr">
+        <is>
+          <t>Thank you for joining us. Tap a photo to see it larger and download the original.</t>
+        </is>
+      </c>
+      <c r="F227" s="8" t="n"/>
+      <c r="G227" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H227" s="10" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="inlineStr">
+        <is>
+          <t>photos.empty</t>
+        </is>
+      </c>
+      <c r="B228" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C228" s="8" t="inlineStr">
+        <is>
+          <t>Kosong</t>
+        </is>
+      </c>
+      <c r="D228" s="10" t="inlineStr">
+        <is>
+          <t>Foto acara sedang kami pilih. Kembali lagi dalam beberapa hari.</t>
+        </is>
+      </c>
+      <c r="E228" s="10" t="inlineStr">
+        <is>
+          <t>We're still choosing the photos. Please check back in a few days.</t>
+        </is>
+      </c>
+      <c r="F228" s="8" t="n"/>
+      <c r="G228" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H228" s="10" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="8" t="inlineStr">
+        <is>
+          <t>photos.closed</t>
+        </is>
+      </c>
+      <c r="B229" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="inlineStr">
+        <is>
+          <t>Tutup</t>
+        </is>
+      </c>
+      <c r="D229" s="10" t="inlineStr">
+        <is>
+          <t>Galeri acara ini sudah ditutup. Hubungi panitia bila Anda membutuhkan foto tertentu.</t>
+        </is>
+      </c>
+      <c r="E229" s="10" t="inlineStr">
+        <is>
+          <t>This gallery has closed. Please contact the organisers if you need a particular photo.</t>
+        </is>
+      </c>
+      <c r="F229" s="8" t="n"/>
+      <c r="G229" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H229" s="10" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="8" t="inlineStr">
+        <is>
+          <t>photos.remove</t>
+        </is>
+      </c>
+      <c r="B230" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C230" s="8" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D230" s="10" t="inlineStr">
+        <is>
+          <t>Minta foto ini dihapus</t>
+        </is>
+      </c>
+      <c r="E230" s="10" t="inlineStr">
+        <is>
+          <t>Ask us to remove this photo</t>
+        </is>
+      </c>
+      <c r="F230" s="8" t="n"/>
+      <c r="G230" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H230" s="10" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="8" t="inlineStr">
+        <is>
+          <t>photos.removeMessage</t>
+        </is>
+      </c>
+      <c r="B231" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C231" s="8" t="inlineStr">
+        <is>
+          <t>Pesan WhatsApp</t>
+        </is>
+      </c>
+      <c r="D231" s="10" t="inlineStr">
+        <is>
+          <t>Halo, saya ingin meminta foto nomor {n} di galeri "{acara}" dihapus. {tautan}</t>
+        </is>
+      </c>
+      <c r="E231" s="10" t="inlineStr">
+        <is>
+          <t>Hello, please remove photo number {n} from the "{event}" gallery. {link}</t>
+        </is>
+      </c>
+      <c r="F231" s="8" t="n"/>
+      <c r="G231" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H231" s="10" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="8" t="inlineStr">
+        <is>
+          <t>photos.back</t>
+        </is>
+      </c>
+      <c r="B232" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C232" s="8" t="inlineStr">
+        <is>
+          <t>Tautan</t>
+        </is>
+      </c>
+      <c r="D232" s="10" t="inlineStr">
+        <is>
+          <t>Kembali ke undangan</t>
+        </is>
+      </c>
+      <c r="E232" s="10" t="inlineStr">
+        <is>
+          <t>Back to the invitation</t>
+        </is>
+      </c>
+      <c r="F232" s="8" t="n"/>
+      <c r="G232" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H232" s="10" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="8" t="inlineStr">
+        <is>
+          <t>photos.count</t>
+        </is>
+      </c>
+      <c r="B233" s="8" t="inlineStr">
+        <is>
+          <t>Galeri</t>
+        </is>
+      </c>
+      <c r="C233" s="8" t="inlineStr">
+        <is>
+          <t>Jumlah</t>
+        </is>
+      </c>
+      <c r="D233" s="10" t="inlineStr">
+        <is>
+          <t>{n} foto</t>
+        </is>
+      </c>
+      <c r="E233" s="10" t="inlineStr">
+        <is>
+          <t>{n} photos</t>
+        </is>
+      </c>
+      <c r="F233" s="8" t="n"/>
+      <c r="G233" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H233" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G233" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: tambah tiket QR tamu dan check-in di pintu masuk
- Tiket untuk tamu undangan personal yang hadir: nama, jumlah orang, dan QR
- Simpan tiket sebagai gambar, PDF, atau kirim ke WhatsApp sendiri
- Tab Check-in: pindai QR dengan kamera, cari nama, dan batalkan check-in yang salah
- QR membuka halaman konfirmasi untuk panitia yang login, sehingga kamera ponsel biasa pun bisa dipakai
- Hasil pindai menampilkan jumlah orang, alergi, dan akses; pindai ulang tidak menggandakan
- Migrasi 202610210003_tickets_checkin.sql beserta uji SQL lokal

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H233"/>
+  <dimension ref="A1:H240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8729,10 +8729,248 @@
       </c>
       <c r="H233" s="10" t="n"/>
     </row>
+    <row r="234">
+      <c r="A234" s="8" t="inlineStr">
+        <is>
+          <t>ticket.title</t>
+        </is>
+      </c>
+      <c r="B234" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C234" s="8" t="inlineStr">
+        <is>
+          <t>Judul halaman</t>
+        </is>
+      </c>
+      <c r="D234" s="10" t="inlineStr">
+        <is>
+          <t>Tiket masuk</t>
+        </is>
+      </c>
+      <c r="E234" s="10" t="inlineStr">
+        <is>
+          <t>Entry ticket</t>
+        </is>
+      </c>
+      <c r="F234" s="8" t="n"/>
+      <c r="G234" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H234" s="10" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="8" t="inlineStr">
+        <is>
+          <t>ticket.view</t>
+        </is>
+      </c>
+      <c r="B235" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C235" s="8" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D235" s="10" t="inlineStr">
+        <is>
+          <t>Lihat tiket masuk</t>
+        </is>
+      </c>
+      <c r="E235" s="10" t="inlineStr">
+        <is>
+          <t>View your entry ticket</t>
+        </is>
+      </c>
+      <c r="F235" s="8" t="n"/>
+      <c r="G235" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H235" s="10" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="8" t="inlineStr">
+        <is>
+          <t>ticket.party</t>
+        </is>
+      </c>
+      <c r="B236" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C236" s="8" t="inlineStr">
+        <is>
+          <t>Jumlah orang</t>
+        </is>
+      </c>
+      <c r="D236" s="10" t="inlineStr">
+        <is>
+          <t>Untuk {n} orang</t>
+        </is>
+      </c>
+      <c r="E236" s="10" t="inlineStr">
+        <is>
+          <t>For {n} people</t>
+        </is>
+      </c>
+      <c r="F236" s="8" t="n"/>
+      <c r="G236" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H236" s="10" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="8" t="inlineStr">
+        <is>
+          <t>ticket.notYet</t>
+        </is>
+      </c>
+      <c r="B237" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C237" s="8" t="inlineStr">
+        <is>
+          <t>Belum hadir</t>
+        </is>
+      </c>
+      <c r="D237" s="10" t="inlineStr">
+        <is>
+          <t>Tiket muncul setelah Anda mengonfirmasi hadir.</t>
+        </is>
+      </c>
+      <c r="E237" s="10" t="inlineStr">
+        <is>
+          <t>Your ticket appears once you confirm you're coming.</t>
+        </is>
+      </c>
+      <c r="F237" s="8" t="n"/>
+      <c r="G237" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H237" s="10" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="8" t="inlineStr">
+        <is>
+          <t>ticket.unavailable</t>
+        </is>
+      </c>
+      <c r="B238" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C238" s="8" t="inlineStr">
+        <is>
+          <t>Belum tersedia</t>
+        </is>
+      </c>
+      <c r="D238" s="10" t="inlineStr">
+        <is>
+          <t>Tiket belum tersedia untuk acara ini. Cukup sebutkan nama Anda di meja registrasi.</t>
+        </is>
+      </c>
+      <c r="E238" s="10" t="inlineStr">
+        <is>
+          <t>Tickets aren't available for this event yet. Just give your name at the registration desk.</t>
+        </is>
+      </c>
+      <c r="F238" s="8" t="n"/>
+      <c r="G238" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H238" s="10" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="8" t="inlineStr">
+        <is>
+          <t>ticket.whatsappMessage</t>
+        </is>
+      </c>
+      <c r="B239" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C239" s="8" t="inlineStr">
+        <is>
+          <t>Pesan WhatsApp</t>
+        </is>
+      </c>
+      <c r="D239" s="10" t="inlineStr">
+        <is>
+          <t>Tiket masuk saya untuk {acara}: {tautan}</t>
+        </is>
+      </c>
+      <c r="E239" s="10" t="inlineStr">
+        <is>
+          <t>My entry ticket for {event}: {link}</t>
+        </is>
+      </c>
+      <c r="F239" s="8" t="n"/>
+      <c r="G239" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H239" s="10" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="8" t="inlineStr">
+        <is>
+          <t>ticket.private</t>
+        </is>
+      </c>
+      <c r="B240" s="8" t="inlineStr">
+        <is>
+          <t>Tiket</t>
+        </is>
+      </c>
+      <c r="C240" s="8" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D240" s="10" t="inlineStr">
+        <is>
+          <t>Tiket ini khusus untuk Anda. Jangan bagikan ke orang lain.</t>
+        </is>
+      </c>
+      <c r="E240" s="10" t="inlineStr">
+        <is>
+          <t>This ticket is just for you. Please don't share it.</t>
+        </is>
+      </c>
+      <c r="F240" s="8" t="n"/>
+      <c r="G240" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H240" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G233" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: E-Guide, buku panduan digital untuk tamu, dengan modul per jenis acara
- Jenis acara baru "eguide" dan templat "E-Guide destinasi": sampul,
  bab tulisan sendiri (cerita, kartu tempat, daftar frasa, tips), dan
  urutan baca bersama nuansa acara, jadwal, lokasi beserta rute dan
  galeri, persiapan, serta kontak.
- Halaman tamu dibaca per halaman seperti buku: daftar isi, sebelumnya/
  berikutnya, geser di HP, tautan per bab, dan unduh PDF seluruh buku.
  Bahasa dipilih per E-Guide (ID, EN, atau keduanya).
- Setiap jenis acara hanya menawarkan modul yang cocok; kartu tetap
  seperti sebelumnya.
- Pratinjau editor E-Guide menampilkan buku, bukan undangan.
- Migrasi 202610260001: E-Guide bisa dipublikasikan tanpa syarat
  undangan (penyelenggara, pengantar, lokasi).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H240"/>
+  <dimension ref="A1:H265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8967,10 +8967,860 @@
       </c>
       <c r="H240" s="10" t="n"/>
     </row>
+    <row r="241">
+      <c r="A241" s="8" t="inlineStr">
+        <is>
+          <t>guide.eyebrow</t>
+        </is>
+      </c>
+      <c r="B241" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C241" s="8" t="inlineStr">
+        <is>
+          <t>Sampul</t>
+        </is>
+      </c>
+      <c r="D241" s="10" t="inlineStr">
+        <is>
+          <t>Panduan digital</t>
+        </is>
+      </c>
+      <c r="E241" s="10" t="inlineStr">
+        <is>
+          <t>Digital guide</t>
+        </is>
+      </c>
+      <c r="F241" s="8" t="n"/>
+      <c r="G241" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H241" s="10" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="8" t="inlineStr">
+        <is>
+          <t>guide.start</t>
+        </is>
+      </c>
+      <c r="B242" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C242" s="8" t="inlineStr">
+        <is>
+          <t>Tombol di sampul</t>
+        </is>
+      </c>
+      <c r="D242" s="10" t="inlineStr">
+        <is>
+          <t>Mulai membaca</t>
+        </is>
+      </c>
+      <c r="E242" s="10" t="inlineStr">
+        <is>
+          <t>Start reading</t>
+        </is>
+      </c>
+      <c r="F242" s="8" t="n"/>
+      <c r="G242" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H242" s="10" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="8" t="inlineStr">
+        <is>
+          <t>guide.toc</t>
+        </is>
+      </c>
+      <c r="B243" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C243" s="8" t="inlineStr">
+        <is>
+          <t>Judul daftar isi dan tombol kembali ke daftar isi</t>
+        </is>
+      </c>
+      <c r="D243" s="10" t="inlineStr">
+        <is>
+          <t>Daftar isi</t>
+        </is>
+      </c>
+      <c r="E243" s="10" t="inlineStr">
+        <is>
+          <t>Contents</t>
+        </is>
+      </c>
+      <c r="F243" s="8" t="n"/>
+      <c r="G243" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H243" s="10" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="8" t="inlineStr">
+        <is>
+          <t>guide.prev</t>
+        </is>
+      </c>
+      <c r="B244" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C244" s="8" t="inlineStr">
+        <is>
+          <t>Tombol halaman sebelumnya</t>
+        </is>
+      </c>
+      <c r="D244" s="10" t="inlineStr">
+        <is>
+          <t>Sebelumnya</t>
+        </is>
+      </c>
+      <c r="E244" s="10" t="inlineStr">
+        <is>
+          <t>Previous</t>
+        </is>
+      </c>
+      <c r="F244" s="8" t="n"/>
+      <c r="G244" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H244" s="10" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="8" t="inlineStr">
+        <is>
+          <t>guide.next</t>
+        </is>
+      </c>
+      <c r="B245" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C245" s="8" t="inlineStr">
+        <is>
+          <t>Tombol halaman berikutnya</t>
+        </is>
+      </c>
+      <c r="D245" s="10" t="inlineStr">
+        <is>
+          <t>Berikutnya</t>
+        </is>
+      </c>
+      <c r="E245" s="10" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="F245" s="8" t="n"/>
+      <c r="G245" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H245" s="10" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="8" t="inlineStr">
+        <is>
+          <t>guide.position</t>
+        </is>
+      </c>
+      <c r="B246" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C246" s="8" t="inlineStr">
+        <is>
+          <t>Posisi halaman untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D246" s="10" t="inlineStr">
+        <is>
+          <t>Halaman {n} dari {total}</t>
+        </is>
+      </c>
+      <c r="E246" s="10" t="inlineStr">
+        <is>
+          <t>Page {n} of {total}</t>
+        </is>
+      </c>
+      <c r="F246" s="8" t="n"/>
+      <c r="G246" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H246" s="10" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="8" t="inlineStr">
+        <is>
+          <t>guide.chapter</t>
+        </is>
+      </c>
+      <c r="B247" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C247" s="8" t="inlineStr">
+        <is>
+          <t>Label kecil di atas judul halaman</t>
+        </is>
+      </c>
+      <c r="D247" s="10" t="inlineStr">
+        <is>
+          <t>Bab {n}</t>
+        </is>
+      </c>
+      <c r="E247" s="10" t="inlineStr">
+        <is>
+          <t>Chapter {n}</t>
+        </is>
+      </c>
+      <c r="F247" s="8" t="n"/>
+      <c r="G247" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H247" s="10" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="8" t="inlineStr">
+        <is>
+          <t>guide.pdf</t>
+        </is>
+      </c>
+      <c r="B248" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C248" s="8" t="inlineStr">
+        <is>
+          <t>Tombol unduh</t>
+        </is>
+      </c>
+      <c r="D248" s="10" t="inlineStr">
+        <is>
+          <t>Unduh PDF</t>
+        </is>
+      </c>
+      <c r="E248" s="10" t="inlineStr">
+        <is>
+          <t>Download PDF</t>
+        </is>
+      </c>
+      <c r="F248" s="8" t="n"/>
+      <c r="G248" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H248" s="10" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="8" t="inlineStr">
+        <is>
+          <t>guide.pdf.preparing</t>
+        </is>
+      </c>
+      <c r="B249" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C249" s="8" t="inlineStr">
+        <is>
+          <t>Tombol unduh saat menunggu foto</t>
+        </is>
+      </c>
+      <c r="D249" s="10" t="inlineStr">
+        <is>
+          <t>Menyiapkan PDF…</t>
+        </is>
+      </c>
+      <c r="E249" s="10" t="inlineStr">
+        <is>
+          <t>Preparing the PDF…</t>
+        </is>
+      </c>
+      <c r="F249" s="8" t="n"/>
+      <c r="G249" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H249" s="10" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="8" t="inlineStr">
+        <is>
+          <t>guide.pdf.hint</t>
+        </is>
+      </c>
+      <c r="B250" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C250" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah tombol unduh</t>
+        </is>
+      </c>
+      <c r="D250" s="10" t="inlineStr">
+        <is>
+          <t>Di jendela cetak, pilih “Simpan sebagai PDF”.</t>
+        </is>
+      </c>
+      <c r="E250" s="10" t="inlineStr">
+        <is>
+          <t>In the print window, choose “Save as PDF”.</t>
+        </is>
+      </c>
+      <c r="F250" s="8" t="n"/>
+      <c r="G250" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H250" s="10" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="8" t="inlineStr">
+        <is>
+          <t>guide.part.experience</t>
+        </is>
+      </c>
+      <c r="B251" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C251" s="8" t="inlineStr">
+        <is>
+          <t>Daftar isi: bagian pengalaman</t>
+        </is>
+      </c>
+      <c r="D251" s="10" t="inlineStr">
+        <is>
+          <t>Nuansa acara</t>
+        </is>
+      </c>
+      <c r="E251" s="10" t="inlineStr">
+        <is>
+          <t>The experience</t>
+        </is>
+      </c>
+      <c r="F251" s="8" t="n"/>
+      <c r="G251" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H251" s="10" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="8" t="inlineStr">
+        <is>
+          <t>guide.part.agenda</t>
+        </is>
+      </c>
+      <c r="B252" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C252" s="8" t="inlineStr">
+        <is>
+          <t>Daftar isi: bagian jadwal</t>
+        </is>
+      </c>
+      <c r="D252" s="10" t="inlineStr">
+        <is>
+          <t>Jadwal</t>
+        </is>
+      </c>
+      <c r="E252" s="10" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="F252" s="8" t="n"/>
+      <c r="G252" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H252" s="10" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="8" t="inlineStr">
+        <is>
+          <t>guide.part.location</t>
+        </is>
+      </c>
+      <c r="B253" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C253" s="8" t="inlineStr">
+        <is>
+          <t>Daftar isi: bagian lokasi</t>
+        </is>
+      </c>
+      <c r="D253" s="10" t="inlineStr">
+        <is>
+          <t>Lokasi &amp; rute</t>
+        </is>
+      </c>
+      <c r="E253" s="10" t="inlineStr">
+        <is>
+          <t>Location &amp; route</t>
+        </is>
+      </c>
+      <c r="F253" s="8" t="n"/>
+      <c r="G253" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H253" s="10" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="8" t="inlineStr">
+        <is>
+          <t>guide.part.prepare</t>
+        </is>
+      </c>
+      <c r="B254" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C254" s="8" t="inlineStr">
+        <is>
+          <t>Daftar isi: bagian persiapan</t>
+        </is>
+      </c>
+      <c r="D254" s="10" t="inlineStr">
+        <is>
+          <t>Persiapan</t>
+        </is>
+      </c>
+      <c r="E254" s="10" t="inlineStr">
+        <is>
+          <t>Before you go</t>
+        </is>
+      </c>
+      <c r="F254" s="8" t="n"/>
+      <c r="G254" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H254" s="10" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="8" t="inlineStr">
+        <is>
+          <t>guide.part.contact</t>
+        </is>
+      </c>
+      <c r="B255" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C255" s="8" t="inlineStr">
+        <is>
+          <t>Daftar isi: bagian kontak</t>
+        </is>
+      </c>
+      <c r="D255" s="10" t="inlineStr">
+        <is>
+          <t>Kontak</t>
+        </is>
+      </c>
+      <c r="E255" s="10" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="F255" s="8" t="n"/>
+      <c r="G255" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H255" s="10" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="8" t="inlineStr">
+        <is>
+          <t>guide.story.points</t>
+        </is>
+      </c>
+      <c r="B256" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C256" s="8" t="inlineStr">
+        <is>
+          <t>Bab cerita: judul daftar poin</t>
+        </is>
+      </c>
+      <c r="D256" s="10" t="inlineStr">
+        <is>
+          <t>Yang akan Anda dapat</t>
+        </is>
+      </c>
+      <c r="E256" s="10" t="inlineStr">
+        <is>
+          <t>What awaits you</t>
+        </is>
+      </c>
+      <c r="F256" s="8" t="n"/>
+      <c r="G256" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H256" s="10" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="8" t="inlineStr">
+        <is>
+          <t>guide.map</t>
+        </is>
+      </c>
+      <c r="B257" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C257" s="8" t="inlineStr">
+        <is>
+          <t>Kartu tempat: tombol peta</t>
+        </is>
+      </c>
+      <c r="D257" s="10" t="inlineStr">
+        <is>
+          <t>Buka peta</t>
+        </is>
+      </c>
+      <c r="E257" s="10" t="inlineStr">
+        <is>
+          <t>Open map</t>
+        </is>
+      </c>
+      <c r="F257" s="8" t="n"/>
+      <c r="G257" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H257" s="10" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="8" t="inlineStr">
+        <is>
+          <t>guide.phrase</t>
+        </is>
+      </c>
+      <c r="B258" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C258" s="8" t="inlineStr">
+        <is>
+          <t>Daftar frasa: kolom kiri</t>
+        </is>
+      </c>
+      <c r="D258" s="10" t="inlineStr">
+        <is>
+          <t>Frasa</t>
+        </is>
+      </c>
+      <c r="E258" s="10" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="F258" s="8" t="n"/>
+      <c r="G258" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H258" s="10" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="8" t="inlineStr">
+        <is>
+          <t>guide.meaning</t>
+        </is>
+      </c>
+      <c r="B259" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C259" s="8" t="inlineStr">
+        <is>
+          <t>Daftar frasa: kolom kanan</t>
+        </is>
+      </c>
+      <c r="D259" s="10" t="inlineStr">
+        <is>
+          <t>Arti</t>
+        </is>
+      </c>
+      <c r="E259" s="10" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="F259" s="8" t="n"/>
+      <c r="G259" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H259" s="10" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="8" t="inlineStr">
+        <is>
+          <t>guide.end.label</t>
+        </is>
+      </c>
+      <c r="B260" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C260" s="8" t="inlineStr">
+        <is>
+          <t>Penanda halaman penutup</t>
+        </is>
+      </c>
+      <c r="D260" s="10" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="E260" s="10" t="inlineStr">
+        <is>
+          <t>The end</t>
+        </is>
+      </c>
+      <c r="F260" s="8" t="n"/>
+      <c r="G260" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H260" s="10" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="8" t="inlineStr">
+        <is>
+          <t>guide.end.title</t>
+        </is>
+      </c>
+      <c r="B261" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C261" s="8" t="inlineStr">
+        <is>
+          <t>Halaman penutup: judul</t>
+        </is>
+      </c>
+      <c r="D261" s="10" t="inlineStr">
+        <is>
+          <t>Selamat menikmati perjalanan</t>
+        </is>
+      </c>
+      <c r="E261" s="10" t="inlineStr">
+        <is>
+          <t>Enjoy your journey</t>
+        </is>
+      </c>
+      <c r="F261" s="8" t="n"/>
+      <c r="G261" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H261" s="10" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="8" t="inlineStr">
+        <is>
+          <t>guide.end.text</t>
+        </is>
+      </c>
+      <c r="B262" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C262" s="8" t="inlineStr">
+        <is>
+          <t>Halaman penutup: teks</t>
+        </is>
+      </c>
+      <c r="D262" s="10" t="inlineStr">
+        <is>
+          <t>Simpan panduan ini sebagai PDF agar tetap bisa dibaca tanpa sinyal.</t>
+        </is>
+      </c>
+      <c r="E262" s="10" t="inlineStr">
+        <is>
+          <t>Save this guide as a PDF so you can read it without a signal.</t>
+        </is>
+      </c>
+      <c r="F262" s="8" t="n"/>
+      <c r="G262" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H262" s="10" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="8" t="inlineStr">
+        <is>
+          <t>guide.restart</t>
+        </is>
+      </c>
+      <c r="B263" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C263" s="8" t="inlineStr">
+        <is>
+          <t>Halaman penutup: tombol</t>
+        </is>
+      </c>
+      <c r="D263" s="10" t="inlineStr">
+        <is>
+          <t>Kembali ke awal</t>
+        </is>
+      </c>
+      <c r="E263" s="10" t="inlineStr">
+        <is>
+          <t>Back to the start</t>
+        </is>
+      </c>
+      <c r="F263" s="8" t="n"/>
+      <c r="G263" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H263" s="10" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="8" t="inlineStr">
+        <is>
+          <t>guide.empty</t>
+        </is>
+      </c>
+      <c r="B264" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C264" s="8" t="inlineStr">
+        <is>
+          <t>Sampul, bila belum ada bab</t>
+        </is>
+      </c>
+      <c r="D264" s="10" t="inlineStr">
+        <is>
+          <t>Isi panduan ini sedang disiapkan.</t>
+        </is>
+      </c>
+      <c r="E264" s="10" t="inlineStr">
+        <is>
+          <t>This guide is still being prepared.</t>
+        </is>
+      </c>
+      <c r="F264" s="8" t="n"/>
+      <c r="G264" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H264" s="10" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="8" t="inlineStr">
+        <is>
+          <t>guide.pager.label</t>
+        </is>
+      </c>
+      <c r="B265" s="8" t="inlineStr">
+        <is>
+          <t>E-Guide</t>
+        </is>
+      </c>
+      <c r="C265" s="8" t="inlineStr">
+        <is>
+          <t>Navigasi halaman untuk pembaca layar</t>
+        </is>
+      </c>
+      <c r="D265" s="10" t="inlineStr">
+        <is>
+          <t>Pindah halaman</t>
+        </is>
+      </c>
+      <c r="E265" s="10" t="inlineStr">
+        <is>
+          <t>Turn the page</t>
+        </is>
+      </c>
+      <c r="F265" s="8" t="n"/>
+      <c r="G265" s="10" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+      <c r="H265" s="10" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G240" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G265" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Draf,Perlu diubah,Disetujui"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: templat Handbook trip dengan tema Keraton, bagian transportasi, hotel, do & don't, dan kontak bantuan
Handbook peserta trip beberapa hari (pertama: Surya Madistrindo, Yogyakarta, 5-8 November 2026).
Bagian baru disimpan di content.trip, hanya untuk Program, dan tampil setelah diisi. Data SM dari
deck handbook ada di src/lib/fixtures dan /dev-preview/handbook. Migration memperbarui daftar
templat yang boleh ditawarkan super admin (termasuk panduan-lokasi yang belum ada).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H265"/>
+  <dimension ref="A1:H295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9816,6 +9816,966 @@
         </is>
       </c>
       <c r="H265" s="10" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>nav.transport</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Menu atas</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Transportasi</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Getting there</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>nav.stay</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Menu atas</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>nav.guidelines</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Menu atas</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Panduan</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Good to know</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>nav.contacts</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Menu atas</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Kontak bantuan</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>section.transport.title</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Judul bila kosong</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Informasi perjalanan</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Travel details</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>section.stay.title</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Judul bila kosong</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Tempat menginap</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Where you stay</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>section.guidelines.title</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Trip: do &amp; don't</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Judul bila kosong</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Panduan selama kegiatan</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>During the trip</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>section.contacts.title</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Trip: kontak bantuan</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Judul bila kosong</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Kontak bantuan</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Who to call</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>trip.mode.train</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Label jenis</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Kereta</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Train</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>trip.mode.flight</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Label jenis</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Pesawat</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Flight</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>trip.mode.bus</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Label jenis</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>trip.mode.car</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Label jenis</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Mobil</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Car</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>trip.mode.boat</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Label jenis</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Kapal</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>trip.to</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Pembaca layar, di antara asal dan tujuan</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>ke</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>trip.departs</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Label jam</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Berangkat</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Departs</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>trip.arrives</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Label jam</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Tiba</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Arrives</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>trip.seat</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Kursi &amp; bagasi</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Seats &amp; baggage</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>trip.meeting</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Titik kumpul</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Meeting point</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>trip.meetingTime</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Trip: transportasi</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Jam kumpul</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Meeting time</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>stay.hotel</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Label kecil di atas nama</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>stay.checkIn</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Check-in</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Check-in</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>stay.checkOut</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Check-out</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Check-out</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>stay.breakfast</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Sarapan</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>stay.meeting</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Titik kumpul harian</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Daily meeting point</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>stay.directions</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Tautan</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Petunjuk arah</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Directions</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>stay.call</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Trip: hotel</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Tautan</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Telepon hotel</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Call the hotel</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>guidelines.weather</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Trip: do &amp; don't</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Judul kartu</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Cuaca</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>guidelines.do</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Trip: do &amp; don't</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Judul daftar</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Yang dianjurkan</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Please do</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>guidelines.dont</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Trip: do &amp; don't</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Judul daftar</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Yang perlu dihindari</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Please avoid</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>contacts.call</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Trip: kontak bantuan</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Pembaca layar</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Telepon</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Call</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H142"/>

</xml_diff>

<commit_message>
fix: label acara Program menjadi "Panduan peserta" (Participant guide), bukan undangan
Dipakai di pembuka halaman, kartu pratinjau tautan, dan miniatur templat.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -807,15 +807,19 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Undangan program</t>
+          <t>Panduan peserta</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Programme invitation</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr"/>
+          <t>Participant guide</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Sebelumnya: Undangan program</t>
+        </is>
+      </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Draf</t>

</xml_diff>

<commit_message>
feat: logo klien di kepala halaman tamu, dan kaki halaman "Diselenggarakan oleh" serta "Journey by Werkudara Group"
- Acara bisa memakai logo klien (mis. PT Surya Madistrindo) di kepala halaman menggantikan logo Werkudara; diisi di Identitas & undangan.
- Kaki halaman menyebut penyelenggara dengan label "Diselenggarakan oleh", dan baris paling bawah "Journey by Werkudara Group".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H302"/>
+  <dimension ref="A1:H305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11000,6 +11000,102 @@
         </is>
       </c>
       <c r="G302" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>nav.brandBack</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Navigasi</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Pembaca layar, logo di kepala halaman</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>kembali ke awal halaman</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>back to the top of the page</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>footer.organizedBy</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Label di atas nama penyelenggara</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Diselenggarakan oleh</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Organised by</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>footer.brand</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Baris paling bawah</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Journey by Werkudara Group</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Journey by Werkudara Group</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
feat: handbook lebih lega di desktop, sampul hari sebagai banner, dan keterangan kegiatan tampil langsung (FYI)
- Program di layar lebar: label bagian di atas judul, isi selebar halaman; kartu perjalanan, do & don't, kontak, dan persiapan berdampingan; kolom jam jadwal lebih ramping.
- Gambar per hari tampil sebagai banner 12:5 seperti sampul Facebook/LinkedIn.
- Keterangan kegiatan tidak lagi di balik tombol: kotak "FYI" dengan cuplikan sebagai kalimat pembuka langsung tampil. Cerita panjang tetap lewat "Selengkapnya".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H305"/>
+  <dimension ref="A1:H306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11096,6 +11096,43 @@
         </is>
       </c>
       <c r="G305" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>detail.fyi</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Jadwal per hari</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Label kotak keterangan kegiatan (pengganti Tahukah Anda?)</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>FYI</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>FYI</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Revisi 30 Okt: tampil langsung tanpa tombol</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
fix: keterangan kegiatan tanpa label FYI: ikon lampu, cuplikan tebal, lalu isinya
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H306"/>
+  <dimension ref="A1:H305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11096,43 +11096,6 @@
         </is>
       </c>
       <c r="G305" t="inlineStr">
-        <is>
-          <t>Draf</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>detail.fyi</t>
-        </is>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>Jadwal per hari</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Label kotak keterangan kegiatan (pengganti Tahukah Anda?)</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>FYI</t>
-        </is>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>FYI</t>
-        </is>
-      </c>
-      <c r="F306" t="inlineStr">
-        <is>
-          <t>Revisi 30 Okt: tampil langsung tanpa tombol</t>
-        </is>
-      </c>
-      <c r="G306" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
feat: kartu hotel dengan foto latar dan panel blur, foto kegiatan kecil di samping judul yang bisa dibuka penuh
- Hotel: foto pertama mengisi kartu, info hotel di atas panel kaca buram agar tetap terbaca; foto lain jadi gambar kecil.
- Jadwal: foto tempat tampil kecil di kanan judul kegiatan; ketuk untuk melihat foto penuh (dialog, tutup dengan Esc atau tombol).
- Kartu persiapan: gambar jadi ubin yang bisa dibuka penuh; gambar potongan (tanpa latar) duduk langsung di kartu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H305"/>
+  <dimension ref="A1:H307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11096,6 +11096,70 @@
         </is>
       </c>
       <c r="G305" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>photo.open</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Pembaca layar, gambar kecil yang bisa diperbesar</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Lihat foto penuh: {nama}</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>View full photo: {name}</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>photo.close</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Tombol tutup foto penuh</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Tutup</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
fix: nomor telepon tidak ditampilkan; kontak, hotel, dan rumah sakit memakai tombol Telepon dan WhatsApp
Nomor tetap terlihat di aplikasi telepon saat tombol diketuk. Tombol Telepon dan WhatsApp sejajar satu baris.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H307"/>
+  <dimension ref="A1:H308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11160,6 +11160,38 @@
         </is>
       </c>
       <c r="G307" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>contacts.callHospital</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Trip: kontak bantuan</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Tombol telepon rumah sakit</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Telepon rumah sakit</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Call the hospital</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
feat: kartu handbook seragam, keterangan kegiatan bisa dibuka-tutup, kaki halaman Werkudara Group lengkap
- Semua kartu trip (transportasi, hotel, do & don't, kontak, rumah sakit) memakai pola yang sama dengan kartu persiapan: judul di kiri, ikon di kanan, keterangan singkat, isi tanpa menjorok.
- Hotel kembali menjadi kartu biasa tanpa foto latar; fotonya jadi gambar kecil yang bisa dibuka penuh.
- "Tahukah Anda?" di jadwal tertutup dengan cuplikan sebagai judul; tamu mengetuk untuk membuka cerita.
- Kaki halaman memuat Werkudara Group seperti di werkudara.com: logo, kantor Yogyakarta dan Bali, tombol email/telepon/website, media sosial, dan hak cipta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H308"/>
+  <dimension ref="A1:H316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11192,6 +11192,262 @@
         </is>
       </c>
       <c r="G308" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>footer.managedBy</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Label di atas Werkudara Group bila penyelenggara pihak lain</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Dikelola oleh</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Managed by</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>footer.contact</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Judul tombol kontak Werkudara</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Hubungi kami</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Contact us</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>footer.email</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>footer.callOffice</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Telepon kantor</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Call the office</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>footer.callMobile</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Tombol</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Telepon seluler</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Call mobile</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>footer.map</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Tautan peta kantor</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Lihat peta</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>View map</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>footer.social</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Pembaca layar, deret media sosial</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Media sosial Werkudara Group</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Werkudara Group on social media</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Draf</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>footer.copyright</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Kaki halaman</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Baris hak cipta</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>© {n} Werkudara Group. Hak cipta dilindungi.</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>© {n} Werkudara Group. All rights reserved.</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
         <is>
           <t>Draf</t>
         </is>

</xml_diff>

<commit_message>
fix: tombol utama merah bata, keterangan kegiatan satu baris dengan Selengkapnya, kaki halaman lebih ringkas
- Tema Keraton: tombol dan tautan memakai merah bata #B8231F (lebih tenang dari #E12B27).
- Judul kotak keterangan dibatasi satu baris dengan titik-titik; "Selengkapnya" / "Tutup" di kanan.
- Kaki halaman: satu alamat kantor pusat yang pendek (tanpa label), kontak sebagai tautan teks dalam grid rapi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wording-draf.xlsx
+++ b/docs/wording-draf.xlsx
@@ -11360,7 +11360,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>footer.map</t>
+          <t>footer.social</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -11370,17 +11370,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Tautan peta kantor</t>
+          <t>Pembaca layar, deret media sosial</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Lihat peta</t>
+          <t>Media sosial Werkudara Group</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>View map</t>
+          <t>Werkudara Group on social media</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
@@ -11392,7 +11392,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>footer.social</t>
+          <t>footer.copyright</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -11402,17 +11402,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Pembaca layar, deret media sosial</t>
+          <t>Baris hak cipta</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Media sosial Werkudara Group</t>
+          <t>© {n} Werkudara Group. Hak cipta dilindungi.</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Werkudara Group on social media</t>
+          <t>© {n} Werkudara Group. All rights reserved.</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -11424,27 +11424,27 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>footer.copyright</t>
+          <t>detail.close</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Kaki halaman</t>
+          <t>Jadwal per hari</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Baris hak cipta</t>
+          <t>Teks pada kotak keterangan yang terbuka</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>© {n} Werkudara Group. Hak cipta dilindungi.</t>
+          <t>Tutup</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>© {n} Werkudara Group. All rights reserved.</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">

</xml_diff>